<commit_message>
feat(organizations): add importance field and import support
Add organization importance (high, medium, low) across backend CRUD, persistence, DTOs, and Excel import.

Support optional Importance column with normalization, validation, default medium for new orgs, and merge-safe behavior.

Extend smoke tests for API create/patch and Excel import scenarios.
</commit_message>
<xml_diff>
--- a/tmp/import-smoke/import-create.xlsx
+++ b/tmp/import-smoke/import-create.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,100 +439,105 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Importance</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Category OLD</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>FLAG</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Founding year</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Size adjusted</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>LinkedIn count</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Cantone</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Postal code</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Email organization</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Name personal contact</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Email personal contact (1)</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Email personal contact (2)</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Main Email personal contact</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Solution type</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Solution keyword 1</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Solution keyword 2</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Solution description</t>
         </is>
@@ -559,7 +564,11 @@
           <t>Additive Manufacturing</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> High </t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -567,42 +576,43 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
         <is>
           <t>Bern</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>hello@smoke-org.example</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Alice Smoke</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>alice@smoke-org.example</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>ops@smoke-org.example</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>alice@smoke-org.example</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>